<commit_message>
new dataset and cluster analysis
</commit_message>
<xml_diff>
--- a/clustering/10 subclusters (factoriescap_s (research) 0 visnorm).xlsx
+++ b/clustering/10 subclusters (factoriescap_s (research) 0 visnorm).xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19830" windowHeight="11775"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12885"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="4">
   <si>
     <t>clust</t>
   </si>
@@ -31,12 +31,6 @@
   </si>
   <si>
     <t>researchersavg_s</t>
-  </si>
-  <si>
-    <t>researchers_s</t>
-  </si>
-  <si>
-    <t>Медианы кластеров</t>
   </si>
 </sst>
 </file>
@@ -59,22 +53,26 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="204"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -97,11 +95,24 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -112,10 +123,25 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -137,16 +163,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>476250</xdr:colOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>466724</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>47625</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>15</xdr:col>
-      <xdr:colOff>212683</xdr:colOff>
-      <xdr:row>19</xdr:row>
-      <xdr:rowOff>19050</xdr:rowOff>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>42685</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>44826</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -169,8 +195,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="5800725" y="47625"/>
-          <a:ext cx="5832433" cy="3590925"/>
+          <a:off x="4762499" y="0"/>
+          <a:ext cx="5062361" cy="3854826"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -467,13 +493,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.28515625" customWidth="1"/>
-    <col min="2" max="3" width="16.140625" customWidth="1"/>
-    <col min="4" max="4" width="18.42578125" customWidth="1"/>
-    <col min="5" max="5" width="15.85546875" customWidth="1"/>
+    <col min="2" max="2" width="20.42578125" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="4" width="18.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -489,25 +514,19 @@
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
         <v>0</v>
       </c>
       <c r="B2" s="3">
-        <v>1070793.730129997</v>
+        <v>162837.21855912951</v>
       </c>
       <c r="C2" s="3">
-        <v>45.999999999999979</v>
+        <v>4.7217391304347807</v>
       </c>
       <c r="D2" s="3">
-        <v>2190.399999999996</v>
-      </c>
-      <c r="E2" s="3">
-        <v>2574.299999999992</v>
+        <v>212.19999999999871</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
@@ -515,16 +534,13 @@
         <v>0</v>
       </c>
       <c r="B3" s="3">
-        <v>2767629.0447099982</v>
+        <v>3025432.4796913038</v>
       </c>
       <c r="C3" s="3">
-        <v>54.499999999999957</v>
+        <v>5.3391304347826063</v>
       </c>
       <c r="D3" s="3">
-        <v>4653.4099999999926</v>
-      </c>
-      <c r="E3" s="3">
-        <v>5187.7999999999947</v>
+        <v>688.9017391304335</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
@@ -532,16 +548,13 @@
         <v>1</v>
       </c>
       <c r="B4" s="3">
-        <v>159716.92475630841</v>
+        <v>801635.29944285634</v>
       </c>
       <c r="C4" s="3">
-        <v>2.7777777777777501</v>
+        <v>33.571428571428569</v>
       </c>
       <c r="D4" s="3">
-        <v>80.360194174752749</v>
-      </c>
-      <c r="E4" s="3">
-        <v>88.669902912615697</v>
+        <v>16103.87142857143</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
@@ -549,16 +562,13 @@
         <v>1</v>
       </c>
       <c r="B5" s="3">
-        <v>3135626.5212902902</v>
+        <v>2011498.296257142</v>
       </c>
       <c r="C5" s="3">
-        <v>7.7012987012986844</v>
+        <v>43.428571428571431</v>
       </c>
       <c r="D5" s="3">
-        <v>416.37961165048029</v>
-      </c>
-      <c r="E5" s="3">
-        <v>461.59223300970251</v>
+        <v>16420.185714285719</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
@@ -566,16 +576,13 @@
         <v>2</v>
       </c>
       <c r="B6" s="3">
-        <v>737279.92048333201</v>
+        <v>976198.38146363525</v>
       </c>
       <c r="C6" s="3">
-        <v>33.166666666666643</v>
+        <v>46.18181818181818</v>
       </c>
       <c r="D6" s="3">
-        <v>15045.5</v>
-      </c>
-      <c r="E6" s="3">
-        <v>17607.833333333328</v>
+        <v>2625.9363636363628</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
@@ -583,16 +590,13 @@
         <v>2</v>
       </c>
       <c r="B7" s="3">
-        <v>1899618.0359333309</v>
+        <v>2636356.2542272718</v>
       </c>
       <c r="C7" s="3">
-        <v>47.166666666666643</v>
+        <v>51.81818181818182</v>
       </c>
       <c r="D7" s="3">
-        <v>17749.383333333331</v>
-      </c>
-      <c r="E7" s="3">
-        <v>20649.999999999989</v>
+        <v>3627.5</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
@@ -600,16 +604,13 @@
         <v>3</v>
       </c>
       <c r="B8" s="3">
-        <v>1057295.046339998</v>
+        <v>1714676.431074999</v>
       </c>
       <c r="C8" s="3">
-        <v>7.1999999999999797</v>
+        <v>56</v>
       </c>
       <c r="D8" s="3">
-        <v>3909.979999999995</v>
-      </c>
-      <c r="E8" s="3">
-        <v>3931.3999999999928</v>
+        <v>24939.875</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
@@ -617,16 +618,13 @@
         <v>3</v>
       </c>
       <c r="B9" s="3">
-        <v>2056976.645919997</v>
+        <v>2915021.2695749989</v>
       </c>
       <c r="C9" s="3">
-        <v>20.199999999999971</v>
+        <v>68.25</v>
       </c>
       <c r="D9" s="3">
-        <v>8136.6399999999967</v>
-      </c>
-      <c r="E9" s="3">
-        <v>8925.1999999999935</v>
+        <v>25690.75</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
@@ -634,16 +632,13 @@
         <v>4</v>
       </c>
       <c r="B10" s="3">
-        <v>411941.4643749973</v>
+        <v>396399.34201922989</v>
       </c>
       <c r="C10" s="3">
-        <v>15.2083333333333</v>
+        <v>22.80769230769231</v>
       </c>
       <c r="D10" s="3">
-        <v>1057.31428571428</v>
-      </c>
-      <c r="E10" s="3">
-        <v>1235.5925925925869</v>
+        <v>1834.0230769230759</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
@@ -651,41 +646,36 @@
         <v>4</v>
       </c>
       <c r="B11" s="3">
-        <v>3485435.6023999979</v>
+        <v>3494599.600007691</v>
       </c>
       <c r="C11" s="3">
-        <v>28.185185185185169</v>
+        <v>23.07692307692308</v>
       </c>
       <c r="D11" s="3">
-        <v>2311.9714285714231</v>
-      </c>
-      <c r="E11" s="3">
-        <v>2564.8214285714212</v>
+        <v>2018.4461538461519</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" s="1" t="s">
+      <c r="A14" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B14" s="1" t="s">
+      <c r="B14" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C14" s="1" t="s">
+      <c r="C14" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D14" s="1" t="s">
+      <c r="D14" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="E14" s="1" t="s">
-        <v>4</v>
-      </c>
+      <c r="E14" s="6"/>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="2"/>
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
       <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
+      <c r="E15" s="7"/>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="2">
@@ -693,27 +683,24 @@
       </c>
       <c r="B16" s="3">
         <f>B3/B2</f>
-        <v>2.5846518959108971</v>
-      </c>
-      <c r="C16" s="3">
+        <v>18.579490035889478</v>
+      </c>
+      <c r="C16" s="10">
         <f t="shared" ref="C16:E24" si="0">C3/C2</f>
-        <v>1.1847826086956519</v>
-      </c>
-      <c r="D16" s="3">
+        <v>1.1307550644567219</v>
+      </c>
+      <c r="D16" s="10">
         <f t="shared" si="0"/>
-        <v>2.1244567202337477</v>
-      </c>
-      <c r="E16" s="3">
-        <f t="shared" si="0"/>
-        <v>2.0152274404692578</v>
-      </c>
+        <v>3.2464737942056443</v>
+      </c>
+      <c r="E16" s="8"/>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="2"/>
       <c r="B17" s="2"/>
       <c r="C17" s="2"/>
       <c r="D17" s="2"/>
-      <c r="E17" s="2"/>
+      <c r="E17" s="7"/>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="2">
@@ -721,23 +708,21 @@
       </c>
       <c r="B18" s="3">
         <f>B5/B4</f>
-        <v>19.632399797795639</v>
-      </c>
-      <c r="C18" s="3">
+        <v>2.5092436643635221</v>
+      </c>
+      <c r="C18" s="10">
         <f t="shared" si="0"/>
-        <v>2.7724675324675538</v>
+        <v>1.2936170212765958</v>
       </c>
       <c r="D18" s="3">
         <f t="shared" si="0"/>
-        <v>5.181416196494169</v>
-      </c>
-      <c r="E18" s="3">
-        <f t="shared" si="0"/>
-        <v>5.2057374356730968</v>
-      </c>
+        <v>1.019642126871001</v>
+      </c>
+      <c r="E18" s="8"/>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="2"/>
+      <c r="E19" s="9"/>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="2">
@@ -745,23 +730,21 @@
       </c>
       <c r="B20" s="3">
         <f>B7/B6</f>
-        <v>2.5765221365150093</v>
-      </c>
-      <c r="C20" s="3">
+        <v>2.7006357563044983</v>
+      </c>
+      <c r="C20" s="10">
         <f t="shared" si="0"/>
-        <v>1.4221105527638194</v>
-      </c>
-      <c r="D20" s="3">
+        <v>1.1220472440944882</v>
+      </c>
+      <c r="D20" s="10">
         <f t="shared" si="0"/>
-        <v>1.1797137571588403</v>
-      </c>
-      <c r="E20" s="3">
-        <f t="shared" si="0"/>
-        <v>1.1727734814997111</v>
-      </c>
+        <v>1.3814119984905822</v>
+      </c>
+      <c r="E20" s="8"/>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="2"/>
+      <c r="E21" s="9"/>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="2">
@@ -769,23 +752,21 @@
       </c>
       <c r="B22" s="3">
         <f>B9/B8</f>
-        <v>1.945508638331904</v>
-      </c>
-      <c r="C22" s="3">
+        <v>1.7000416036204893</v>
+      </c>
+      <c r="C22" s="10">
         <f t="shared" si="0"/>
-        <v>2.8055555555555594</v>
-      </c>
-      <c r="D22" s="3">
+        <v>1.21875</v>
+      </c>
+      <c r="D22" s="10">
         <f t="shared" si="0"/>
-        <v>2.0809927416508542</v>
-      </c>
-      <c r="E22" s="3">
-        <f t="shared" si="0"/>
-        <v>2.2702345220532152</v>
-      </c>
+        <v>1.0301074083170023</v>
+      </c>
+      <c r="E22" s="8"/>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="2"/>
+      <c r="E23" s="9"/>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="2">
@@ -793,131 +774,108 @@
       </c>
       <c r="B24" s="3">
         <f>B11/B10</f>
-        <v>8.4609972625313254</v>
+        <v>8.8158562075467906</v>
       </c>
       <c r="C24" s="3">
         <f t="shared" si="0"/>
-        <v>1.8532724505327276</v>
-      </c>
-      <c r="D24" s="3">
+        <v>1.0118043844856661</v>
+      </c>
+      <c r="D24" s="10">
         <f t="shared" si="0"/>
-        <v>2.186645408852625</v>
-      </c>
-      <c r="E24" s="3">
-        <f t="shared" si="0"/>
-        <v>2.0757824577029673</v>
+        <v>1.1005565738204783</v>
+      </c>
+      <c r="E24" s="8"/>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E25" s="9"/>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A27" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="D27" s="4" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A28" s="5" t="s">
-        <v>5</v>
+      <c r="A28" s="2">
+        <v>0</v>
+      </c>
+      <c r="B28" s="2">
+        <v>377383.36859999882</v>
+      </c>
+      <c r="C28" s="2">
+        <v>4.9999999999999947</v>
+      </c>
+      <c r="D28" s="2">
+        <v>169.99999999999909</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A29" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B29" s="1" t="s">
+      <c r="A29" s="2">
         <v>1</v>
       </c>
-      <c r="C29" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D29" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E29" s="1" t="s">
-        <v>4</v>
+      <c r="B29" s="2">
+        <v>1616706.626599998</v>
+      </c>
+      <c r="C29" s="2">
+        <v>40</v>
+      </c>
+      <c r="D29" s="2">
+        <v>15886.6</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="2">
-        <v>0</v>
-      </c>
-      <c r="B30" s="4">
-        <v>1323628.3493999969</v>
+        <v>2</v>
+      </c>
+      <c r="B30" s="2">
+        <v>1305131.6499999999</v>
       </c>
       <c r="C30" s="2">
-        <v>50.999999999999993</v>
+        <v>50</v>
       </c>
       <c r="D30" s="2">
-        <v>2957</v>
-      </c>
-      <c r="E30" s="2">
-        <v>3335.9999999999941</v>
+        <v>2638.199999999998</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="2">
-        <v>1</v>
-      </c>
-      <c r="B31" s="4">
-        <v>347785.94959999912</v>
+        <v>3</v>
+      </c>
+      <c r="B31" s="2">
+        <v>2567021.7022000002</v>
       </c>
       <c r="C31" s="2">
-        <v>4.9999999999999449</v>
+        <v>65</v>
       </c>
       <c r="D31" s="2">
-        <v>159.449999999997</v>
-      </c>
-      <c r="E31" s="2">
-        <v>191.49999999999289</v>
+        <v>25879.4</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="2">
-        <v>2</v>
-      </c>
-      <c r="B32" s="4">
-        <v>1209456.1932999981</v>
+        <v>4</v>
+      </c>
+      <c r="B32" s="2">
+        <v>663392.6873999997</v>
       </c>
       <c r="C32" s="2">
-        <v>40.499999999999957</v>
+        <v>22.5</v>
       </c>
       <c r="D32" s="2">
-        <v>15830.3</v>
-      </c>
-      <c r="E32" s="2">
-        <v>19196.999999999989</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A33" s="2">
-        <v>3</v>
-      </c>
-      <c r="B33" s="4">
-        <v>1584809.279999997</v>
-      </c>
-      <c r="C33" s="2">
-        <v>9.9999999999999556</v>
-      </c>
-      <c r="D33" s="2">
-        <v>4065.3999999999928</v>
-      </c>
-      <c r="E33" s="2">
-        <v>4351.9999999999955</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A34" s="2">
-        <v>4</v>
-      </c>
-      <c r="B34" s="4">
-        <v>678275.26479999814</v>
-      </c>
-      <c r="C34" s="2">
-        <v>21.999999999999961</v>
-      </c>
-      <c r="D34" s="2">
-        <v>1347.9999999999991</v>
-      </c>
-      <c r="E34" s="2">
-        <v>1561.999999999992</v>
+        <v>1325.9999999999991</v>
       </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="B2:B11">
-    <cfRule type="colorScale" priority="8">
+    <cfRule type="colorScale" priority="6">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -929,7 +887,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C2:C11">
-    <cfRule type="colorScale" priority="7">
+    <cfRule type="colorScale" priority="5">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -941,30 +899,6 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D2:D11">
-    <cfRule type="colorScale" priority="6">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E2:E11">
-    <cfRule type="colorScale" priority="5">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B30:B34">
     <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="min"/>
@@ -976,7 +910,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C30:C34">
+  <conditionalFormatting sqref="B28:B32">
     <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="min"/>
@@ -988,7 +922,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D30:D34">
+  <conditionalFormatting sqref="C28:C32">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
@@ -1000,7 +934,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E30:E34">
+  <conditionalFormatting sqref="D28:D32">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>

</xml_diff>